<commit_message>
Implemented batch 1 of onboarding Test
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="503">
   <si>
     <t>S.No.</t>
   </si>
@@ -90,10 +90,13 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Extends the existing TST_LAND_TC_5 (hero heading/sub-heading/buttons/logo) with the header and footer items — a new function, not a duplicate.</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Not Run</t>
+    <t>Verified on Production: header logo/home link, language switcher, login/signup buttons, heading text, and all footer links are visible.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 1)</t>
   </si>
   <si>
     <t>Automate</t>
@@ -120,6 +123,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_LAND_TC_3 already clicks Log in and checks the login page is launched. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: clicking Log in navigates to the login page (/login).</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 2, Suite 3)</t>
+  </si>
+  <si>
     <t>TST_LAND_TC_2</t>
   </si>
   <si>
@@ -136,6 +145,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_LAND_TC_2 already clicks Sign up and checks the signup page is launched (used by the LP setup chain). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
+  </si>
+  <si>
+    <t>Verified on Production: clicking Sign up opens the role selection screen (/regoptions).</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 4, Suite 5)</t>
   </si>
   <si>
     <t>TST_LAND_TC_7</t>
@@ -164,6 +179,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. The existing TST_LAND_TC_4 only opens the dropdown (asserts the click); this case asserts the outcome. Automation reuses LAND_TC_4 for the click.</t>
   </si>
   <si>
+    <t>Verified on Production: language switcher expands, changes language to Español, and reverts back to English.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_1</t>
   </si>
   <si>
@@ -182,6 +200,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Source row split one case per link. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_1 already clicks the link and checks the page is launched (footer.test.js, active). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: Terms of use page opens with expected heading in the same tab.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_2</t>
   </si>
   <si>
@@ -197,6 +218,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_2 already clicks the link and checks the page is launched (active). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: Privacy notice page opens with expected heading in the same tab.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_3</t>
   </si>
   <si>
@@ -212,6 +236,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_3 already clicks the link and checks the page is launched (active). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: Accessibility page opens with expected heading in the same tab.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_7</t>
   </si>
   <si>
@@ -227,6 +254,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_7 already clicks the link and checks the page is launched (active). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: Cambridge One for schools page opens in the same tab.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_4</t>
   </si>
   <si>
@@ -245,6 +275,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Source row split one case per link. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_4 already is registered but COMMENTED OUT in footer.test.js — re-enable it and make it assert the new tab (ADR-016 tab helpers). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: Our approach link opens Cambridge English site in new tab and refocuses.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_6</t>
   </si>
   <si>
@@ -260,6 +293,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_6 already is registered but COMMENTED OUT in footer.test.js — re-enable it and make it assert the new tab. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: FAQs opens help centre in a new tab and refocuses.</t>
+  </si>
+  <si>
     <t>TST_FOOT_TC_8</t>
   </si>
   <si>
@@ -270,6 +306,59 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_FOOT_TC_8 already is registered but COMMENTED OUT in footer.test.js — re-enable it and make it assert the new tab. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
+  </si>
+  <si>
+    <t>Verified on Production: Help opens help centre in a new tab and refocuses.</t>
+  </si>
+  <si>
+    <t>TST_LAND_TC_8</t>
+  </si>
+  <si>
+    <t>Verify primary login page - {url}/login-primary</t>
+  </si>
+  <si>
+    <t>TC_HOME_007 — Verify primary login page - {url}/login-primary</t>
+  </si>
+  <si>
+    <t>1. Go to the pre-login homepage / navigate to {url}/login-primary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The header shows the Cambridge One logo/home link.
+2. The page shows the Primary-themed background image and the 'Welcome to Cambridge One' heading.
+3. The login area shows the username/email field, the password field, a 'Log in' button and a 'Forgot password' link.
+4. Entering valid credentials and clicking 'Log in' takes the user to their dashboard, while invalid or empty credentials show an error message.
+5. The footer shows 'Terms of use', 'Privacy notice', 'Accessibility', 'Our approach', 'FAQs', 'Cambridge One for schools', the copyright line '© Cambridge University Press &amp; Assessment 2026', and 'Help'.</t>
+  </si>
+  <si>
+    <t>Source: OnboardingApp_Test_Plan.xlsx. Direct entry to the primary-themed login route.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Not Run</t>
+  </si>
+  <si>
+    <t>TST_LAND_TC_9</t>
+  </si>
+  <si>
+    <t>Verify secondary login page - {url}/login-secondary</t>
+  </si>
+  <si>
+    <t>TC_HOME_008 — Verify secondary login page - {url}/login-secondary</t>
+  </si>
+  <si>
+    <t>1. Go to the pre-login homepage / navigate to {url}/login-secondary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The header shows the Cambridge One logo/home link.
+2. The page shows the Secondary-themed background image and the 'Welcome to Cambridge One' heading.
+3. The login area shows the username/email field, the password field, a 'Log in' button and a 'Forgot password' link.
+4. Entering valid credentials and clicking 'Log in' takes the user to their dashboard, while invalid or empty credentials show an error message.
+5. The footer shows 'Terms of use', 'Privacy notice', 'Accessibility', 'Our approach', 'FAQs', 'Cambridge One for schools', the copyright line '© Cambridge University Press &amp; Assessment 2026', and 'Help'.</t>
+  </si>
+  <si>
+    <t>Source: OnboardingApp_Test_Plan.xlsx. Direct entry to the secondary-themed login route.</t>
   </si>
   <si>
     <t>TST_LOGI_TC_5</t>
@@ -325,6 +414,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Side-effect free.</t>
   </si>
   <si>
+    <t>Verified on Production: required-field validation messages displayed for username and password fields on blank submit.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 2)</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_8</t>
   </si>
   <si>
@@ -361,7 +456,7 @@
     <t>TC_LOGIN_004 — Verify the account is temporarily locked after 5 consecutive failed login attempts</t>
   </si>
   <si>
-    <t>A registered, DISPOSABLE test account exists (not used by any other case). User is on the Log in page (homepage → "Log in").</t>
+    <t>A dedicated test account (cqatestuserforblockDND@mailsac.com) exists for lockout testing. User is on the Log in page (homepage → "Log in").</t>
   </si>
   <si>
     <t xml:space="preserve">1. Enter the account's e-mail with an incorrect password and click 'Log in'.
@@ -369,14 +464,14 @@
 3. Try a 6th time with the CORRECT password.</t>
   </si>
   <si>
-    <t>&lt;DISPOSABLE_ACCOUNT_EMAIL&gt;; wrong password ×5, then the correct password. Passwords come from `{{env.*}}` tokens, never plaintext test data (ADR-023).</t>
+    <t>cqatestuserforblockDND@mailsac.com; wrong password ×5, then the correct password. Passwords come from `{{env.*}}` tokens, never plaintext test data (ADR-023).</t>
   </si>
   <si>
     <t xml:space="preserve">1. Each of the first 5 attempts shows the 'check your login and password' alert referencing the 5-attempt limit.
-2. After the 5th failure the account is temporarily locked: the 6th attempt, even with the correct password, is rejected.</t>
-  </si>
-  <si>
-    <t>Source: OnboardingApp_Test_Plan.xlsx. LOCKS AN ACCOUNT — never a shared/pool account (migration plan Q10). Needs a disposable account per run (e.g. one created by the signup suite). Lockout duration and the exact 5th/6th-attempt copy are [ASSUMED] — not stated in the source.</t>
+2. After the 5th failure the account is temporarily locked for 2 minutes: the 6th attempt, even with the correct password, is rejected.</t>
+  </si>
+  <si>
+    <t>Source: OnboardingApp_Test_Plan.xlsx. Account is locked for 2 minutes on 5 consecutive wrong password attempts (user confirmed 2026-09-24). Uses dedicated test user cqatestuserforblockDND@mailsac.com.</t>
   </si>
   <si>
     <t>TST_LOGI_TC_10</t>
@@ -403,6 +498,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. The existing TST_LOGI_TC_3 (login.test.js, not registered in C1TCRepository) only clicks the eye icon; this case asserts the field type. Automation reuses the click.</t>
   </si>
   <si>
+    <t>Verified on Production: password field type changes from password to text and back to password on clicking show password toggle.</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_4</t>
   </si>
   <si>
@@ -419,6 +517,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_LOGI_TC_4 already clicks Forgotten your password and checks the reset page is launched. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
+  </si>
+  <si>
+    <t>Verified on Production: Forgotten your password link navigates to the reset password form.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 3)</t>
   </si>
   <si>
     <t>TST_LOGI_TC_6</t>
@@ -664,6 +768,12 @@
     <t xml:space="preserve">Source: OnboardingApp_Test_Plan.xlsx. </t>
   </si>
   <si>
+    <t>Verified on Production: submitting blank email displays 'This field is required' error message.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 3 via TST_RESE_TC_2)</t>
+  </si>
+  <si>
     <t>TST_RESE_TC_7</t>
   </si>
   <si>
@@ -724,6 +834,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_RESE_TC_4 already clicks Back to login and checks the login page is launched. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
+  </si>
+  <si>
+    <t>Verified on Production: clicking Back to login navigates back to the Login form.</t>
   </si>
   <si>
     <t>TST_RESE_TC_9</t>
@@ -880,6 +993,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. onboarding.md §A1: Next is natively disabled until a role is picked (seen live, thor 2026-09-22).</t>
   </si>
   <si>
+    <t>Verified on Production: Learner, Teacher, and Parent role options are displayed with none pre-selected and Next button disabled.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 4)</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_66</t>
   </si>
   <si>
@@ -905,6 +1024,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. The existing TST_SNUP_TC_59 checks the dialog NAMES the role and then continues; this case asserts the full copy and both buttons and stops at the dialog.</t>
   </si>
   <si>
+    <t>Verified on Production: modal dialog confirms selected role ('You have selected Teacher. Please check this is the right role') with 'Yes, continue' and 'No, go back' buttons.</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_67</t>
   </si>
   <si>
@@ -921,6 +1043,9 @@
     <t>The dialog closes, the user stays on the role-selection page and 'Teacher' is still selected.</t>
   </si>
   <si>
+    <t>Verified on Production: clicking 'No, go back' closes dialog and retains previously selected role.</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_59</t>
   </si>
   <si>
@@ -943,6 +1068,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_SNUP_TC_59 already selects a role, checks the dialog names it, clicks Yes, continue and checks the role's next screen (data: role, expectedScreen) — run it for Parent too. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: clicking 'Yes, continue' on confirmation dialog navigates to the role registration flow (Learner age gate).</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 5 via TST_SNUP_TC_69)</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_68</t>
   </si>
   <si>
@@ -956,6 +1087,9 @@
   </si>
   <si>
     <t>The Log in form is shown.</t>
+  </si>
+  <si>
+    <t>Verified on Production: clicking Login link on role selection page navigates to Login form.</t>
   </si>
   <si>
     <t>TST_SNUP_TC_69</t>
@@ -975,6 +1109,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. URL /learner-age-check (onboarding.md §A2). ⚠️ On thor the first-name box also reported visible on this screen (onboarding.md §A2) — check.</t>
+  </si>
+  <si>
+    <t>Verified on Production: learner age check screen (/learner-age-check) is displayed with Location field and Your age dropdown.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 5)</t>
   </si>
   <si>
     <t>TST_SNUP_TC_70</t>
@@ -1004,6 +1144,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Legend 'Learner age gate': India blocks 13–15 (source: confirmed live). Side-effect free.</t>
   </si>
   <si>
+    <t>Verified on Production: selecting underage (13-15) for India displays 'We\'re sorry' blocked screen and 'Go back' button.</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_71</t>
   </si>
   <si>
@@ -1028,6 +1171,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Legend 'Learner age gate': threshold is location-dependent — India blocks 13–15 / allows 16+; United Kingdom blocks 11–12 / allows 13+ (source: confirmed live). Boundary pairs worth adding in Phase 1: India 15/16, UK 12/13.</t>
+  </si>
+  <si>
+    <t>Verified on Production: age dropdown presents options (18+, 17 down to 5); age options verified on learner age check screen.</t>
   </si>
   <si>
     <t>TST_SNUP_TC_63</t>
@@ -1051,6 +1197,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_SNUP_TC_63 already sets country + age and checks the learner profile form opens (LP setup chain). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
+  </si>
+  <si>
+    <t>Verified on Production: selecting age 16+ (18+) with Location India allows user to proceed to the Learner registration profile form.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB1Test_prod (Suite 5 via TST_SNUP_TC_76 prerequisite)</t>
   </si>
   <si>
     <t>TST_SNUP_TC_72</t>
@@ -1107,6 +1259,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Side-effect free (never submits a valid form).</t>
+  </si>
+  <si>
+    <t>Verified on Production: required-field errors ('This field is required') displayed for First name and Last name on blank form submission.</t>
   </si>
   <si>
     <t>TST_SNUP_TC_73</t>
@@ -1510,12 +1665,15 @@
   <si>
     <t>Role: 'Parent' (source); data-driven for Teacher / Learner</t>
   </si>
+  <si>
+    <t>Verified on Production: clicking Login link on Learner registration form returns user to Login page (/login).</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1527,8 +1685,12 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF155724"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1538,6 +1700,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF3D1A66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -1563,7 +1730,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1571,10 +1738,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1916,7 +2086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2017,14 +2187,14 @@
       <c r="L2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -2032,46 +2202,46 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -2079,46 +2249,46 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -2126,13 +2296,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>18</v>
@@ -2141,31 +2311,31 @@
         <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -2173,13 +2343,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>18</v>
@@ -2191,28 +2361,28 @@
         <v>20</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M6" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -2220,13 +2390,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>18</v>
@@ -2238,28 +2408,28 @@
         <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -2267,13 +2437,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>18</v>
@@ -2285,28 +2455,28 @@
         <v>20</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="M8" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -2314,13 +2484,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>18</v>
@@ -2332,28 +2502,28 @@
         <v>20</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -2361,13 +2531,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>18</v>
@@ -2379,28 +2549,28 @@
         <v>20</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M10" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="M10" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2408,13 +2578,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>18</v>
@@ -2426,28 +2596,28 @@
         <v>20</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M11" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
@@ -2455,13 +2625,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>18</v>
@@ -2473,28 +2643,28 @@
         <v>20</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="M12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -2502,46 +2672,46 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -2549,46 +2719,46 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -2596,46 +2766,46 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="H15" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="N15" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -2643,46 +2813,46 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>114</v>
+        <v>22</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M16" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="M16" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>25</v>
+        <v>129</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -2690,46 +2860,46 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -2737,46 +2907,46 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -2784,13 +2954,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>18</v>
@@ -2799,45 +2969,45 @@
         <v>19</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M19" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="M19" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>25</v>
+        <v>129</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>136</v>
+      <c r="B20" s="2" t="s">
+        <v>154</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>138</v>
+        <v>156</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>18</v>
@@ -2846,45 +3016,45 @@
         <v>19</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>141</v>
+        <v>22</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M20" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="M20" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>144</v>
+        <v>161</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>145</v>
+      <c r="B21" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>18</v>
@@ -2893,125 +3063,125 @@
         <v>19</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>148</v>
+        <v>124</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>149</v>
+        <v>22</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O21" s="3" t="s">
-        <v>144</v>
+        <v>104</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>152</v>
+      <c r="B22" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O22" s="3" t="s">
-        <v>144</v>
+        <v>104</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>160</v>
+      <c r="B23" s="4" t="s">
+        <v>177</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>27</v>
+        <v>104</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -3019,43 +3189,43 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O24" s="4" t="s">
         <v>176</v>
@@ -3065,61 +3235,61 @@
       <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>177</v>
+      <c r="B25" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>91</v>
+        <v>198</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O25" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>184</v>
+      <c r="B26" s="5" t="s">
+        <v>200</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>18</v>
@@ -3128,45 +3298,45 @@
         <v>19</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>91</v>
+        <v>206</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>183</v>
+        <v>207</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O26" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O26" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>190</v>
+      <c r="B27" s="5" t="s">
+        <v>209</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>18</v>
@@ -3175,78 +3345,78 @@
         <v>19</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>22</v>
+        <v>214</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>195</v>
+        <v>118</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>27</v>
+        <v>104</v>
+      </c>
+      <c r="O27" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>197</v>
+      <c r="B28" s="5" t="s">
+        <v>216</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>22</v>
+        <v>221</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>202</v>
+        <v>118</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>27</v>
+        <v>104</v>
+      </c>
+      <c r="O28" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3254,46 +3424,46 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>208</v>
+        <v>22</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>210</v>
+        <v>228</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -3301,46 +3471,46 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>215</v>
+        <v>22</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M30" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="M30" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>25</v>
+        <v>237</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -3348,46 +3518,46 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>218</v>
+        <v>238</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>221</v>
+        <v>241</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>22</v>
+        <v>242</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -3395,46 +3565,46 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>225</v>
+        <v>246</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>226</v>
+        <v>247</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>228</v>
+        <v>248</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>229</v>
+        <v>249</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>91</v>
+        <v>250</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>230</v>
+        <v>251</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -3442,13 +3612,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>231</v>
+        <v>252</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>233</v>
+        <v>254</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>18</v>
@@ -3457,31 +3627,31 @@
         <v>19</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>235</v>
+        <v>255</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>236</v>
+        <v>22</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M33" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="M33" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>25</v>
+        <v>161</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -3489,46 +3659,46 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>242</v>
+        <v>262</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>243</v>
+        <v>263</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>245</v>
+        <v>118</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>246</v>
+        <v>265</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
@@ -3536,46 +3706,46 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>247</v>
+        <v>266</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>241</v>
+        <v>268</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>249</v>
+        <v>269</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
@@ -3583,46 +3753,46 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>254</v>
+        <v>274</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>255</v>
+        <v>275</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>256</v>
+        <v>276</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>257</v>
+        <v>277</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>258</v>
+        <v>278</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>259</v>
+        <v>279</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
@@ -3630,46 +3800,46 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>20</v>
+        <v>284</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>265</v>
+        <v>285</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>22</v>
+        <v>286</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>266</v>
+        <v>287</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>267</v>
+        <v>288</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -3677,46 +3847,46 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>268</v>
+        <v>289</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>271</v>
+        <v>292</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>272</v>
+        <v>293</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>274</v>
+        <v>295</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>275</v>
+        <v>296</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
@@ -3724,46 +3894,46 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>276</v>
+        <v>297</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>278</v>
+        <v>299</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>271</v>
+        <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>279</v>
+        <v>300</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>273</v>
+        <v>22</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>280</v>
+        <v>301</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>203</v>
+        <v>302</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M39" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="M39" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>25</v>
+        <v>304</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -3771,46 +3941,46 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>281</v>
+        <v>305</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>285</v>
+        <v>310</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>286</v>
+        <v>311</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>287</v>
+        <v>312</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M40" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="M40" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>25</v>
+        <v>304</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
@@ -3818,13 +3988,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>288</v>
+        <v>314</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>290</v>
+        <v>316</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>18</v>
@@ -3833,31 +4003,31 @@
         <v>19</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>291</v>
+        <v>317</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>22</v>
+        <v>310</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>292</v>
+        <v>318</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M41" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="M41" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>25</v>
+        <v>304</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
@@ -3865,46 +4035,46 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>293</v>
+        <v>320</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>294</v>
+        <v>321</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>295</v>
+        <v>322</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>296</v>
+        <v>323</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>22</v>
+        <v>324</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>297</v>
+        <v>325</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>298</v>
+        <v>326</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M42" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="M42" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>25</v>
+        <v>328</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -3912,46 +4082,46 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>299</v>
+        <v>329</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>301</v>
+        <v>331</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>303</v>
+        <v>332</v>
       </c>
       <c r="I43" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N43" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="J43" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="L43" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N43" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="O43" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -3959,46 +4129,46 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>307</v>
+        <v>335</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>302</v>
-      </c>
       <c r="H44" s="2" t="s">
-        <v>311</v>
+        <v>338</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>312</v>
+        <v>22</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>313</v>
+        <v>339</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>314</v>
+        <v>340</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M44" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="M44" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>25</v>
+        <v>342</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
@@ -4006,46 +4176,46 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>315</v>
+        <v>343</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>316</v>
+        <v>344</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>317</v>
+        <v>345</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>302</v>
+        <v>346</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>318</v>
+        <v>347</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>319</v>
+        <v>348</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>320</v>
+        <v>349</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>321</v>
+        <v>350</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M45" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="M45" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>25</v>
+        <v>342</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
@@ -4053,46 +4223,46 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>322</v>
+        <v>352</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>323</v>
+        <v>353</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>324</v>
+        <v>354</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>18</v>
+        <v>355</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>325</v>
+        <v>346</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>326</v>
+        <v>356</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>327</v>
+        <v>357</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>328</v>
+        <v>358</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>329</v>
+        <v>359</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M46" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="M46" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>25</v>
+        <v>342</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
@@ -4100,46 +4270,46 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>325</v>
+        <v>346</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>333</v>
+        <v>364</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>334</v>
+        <v>365</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>335</v>
+        <v>366</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>336</v>
+        <v>367</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M47" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="M47" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>25</v>
+        <v>369</v>
       </c>
       <c r="O47" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -4147,46 +4317,46 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>337</v>
+        <v>370</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>338</v>
+        <v>371</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>339</v>
+        <v>372</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>271</v>
+        <v>373</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>340</v>
+        <v>374</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>341</v>
+        <v>375</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>342</v>
+        <v>376</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>343</v>
+        <v>377</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O48" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
@@ -4194,46 +4364,46 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>344</v>
+        <v>378</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>345</v>
+        <v>379</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>346</v>
+        <v>380</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>347</v>
+        <v>373</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>348</v>
+        <v>381</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>349</v>
+        <v>382</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>350</v>
+        <v>383</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M49" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="M49" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>25</v>
+        <v>342</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
@@ -4241,46 +4411,46 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>352</v>
+        <v>386</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>353</v>
+        <v>387</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>354</v>
+        <v>388</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>355</v>
+        <v>389</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>356</v>
+        <v>390</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>357</v>
+        <v>391</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>358</v>
+        <v>392</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
@@ -4288,46 +4458,46 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>359</v>
+        <v>393</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>360</v>
+        <v>394</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>361</v>
+        <v>395</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>362</v>
+        <v>396</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>363</v>
+        <v>397</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>364</v>
+        <v>398</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>365</v>
+        <v>399</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>366</v>
+        <v>400</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O51" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
@@ -4335,46 +4505,46 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>367</v>
+        <v>401</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>368</v>
+        <v>402</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>369</v>
+        <v>403</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>370</v>
+        <v>308</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>371</v>
+        <v>404</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>372</v>
+        <v>405</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>373</v>
+        <v>406</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>374</v>
+        <v>407</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O52" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
@@ -4382,46 +4552,46 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>375</v>
+        <v>408</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>376</v>
+        <v>409</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>377</v>
+        <v>410</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>378</v>
+        <v>411</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>379</v>
+        <v>412</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>22</v>
+        <v>413</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>380</v>
+        <v>414</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>381</v>
+        <v>415</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O53" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
@@ -4429,46 +4599,46 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>382</v>
+        <v>416</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>383</v>
+        <v>417</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>384</v>
+        <v>418</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>385</v>
+        <v>419</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>386</v>
+        <v>420</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>387</v>
+        <v>421</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>388</v>
+        <v>422</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>389</v>
+        <v>423</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
@@ -4476,46 +4646,46 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>390</v>
+        <v>424</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>391</v>
+        <v>425</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>392</v>
+        <v>426</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>393</v>
+        <v>427</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>394</v>
+        <v>428</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>395</v>
+        <v>22</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>396</v>
+        <v>429</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>397</v>
+        <v>430</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.25">
@@ -4523,107 +4693,107 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>399</v>
+        <v>432</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>400</v>
+        <v>433</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>401</v>
+        <v>434</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>402</v>
+        <v>435</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>403</v>
+        <v>436</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>404</v>
+        <v>437</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>405</v>
+        <v>438</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>56</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>406</v>
+      <c r="B57" s="2" t="s">
+        <v>439</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>407</v>
+        <v>440</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>408</v>
+        <v>441</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>20</v>
+        <v>442</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>409</v>
+        <v>443</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>22</v>
+        <v>444</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>410</v>
+        <v>445</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>183</v>
+        <v>446</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O57" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>57</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>411</v>
+      <c r="B58" s="2" t="s">
+        <v>447</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>412</v>
+        <v>448</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>413</v>
+        <v>449</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>18</v>
@@ -4632,45 +4802,45 @@
         <v>19</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>271</v>
+        <v>450</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>414</v>
+        <v>451</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>22</v>
+        <v>452</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>415</v>
+        <v>453</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>183</v>
+        <v>454</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O58" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O58" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>58</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>416</v>
+      <c r="B59" s="5" t="s">
+        <v>455</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>417</v>
+        <v>456</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>418</v>
+        <v>457</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>18</v>
@@ -4679,45 +4849,45 @@
         <v>19</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>271</v>
+        <v>20</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>419</v>
+        <v>458</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>420</v>
+        <v>22</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>421</v>
+        <v>459</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O59" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O59" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>59</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>422</v>
+      <c r="B60" s="5" t="s">
+        <v>460</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>423</v>
+        <v>461</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>424</v>
+        <v>462</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>18</v>
@@ -4726,45 +4896,45 @@
         <v>19</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>425</v>
+        <v>463</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>426</v>
+        <v>464</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O60" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O60" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>60</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>427</v>
+      <c r="B61" s="5" t="s">
+        <v>465</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>428</v>
+        <v>466</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>429</v>
+        <v>467</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>18</v>
@@ -4773,45 +4943,45 @@
         <v>19</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>430</v>
+        <v>308</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>431</v>
+        <v>468</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>432</v>
+        <v>469</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>433</v>
+        <v>470</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O61" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O61" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>61</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>434</v>
+      <c r="B62" s="5" t="s">
+        <v>471</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>435</v>
+        <v>472</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>436</v>
+        <v>473</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>18</v>
@@ -4820,45 +4990,45 @@
         <v>19</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>437</v>
+        <v>308</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>438</v>
+        <v>474</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>439</v>
+        <v>22</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O62" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O62" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>62</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>441</v>
+      <c r="B63" s="5" t="s">
+        <v>476</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>442</v>
+        <v>477</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>18</v>
@@ -4867,45 +5037,45 @@
         <v>19</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>444</v>
+        <v>479</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>446</v>
+        <v>481</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>447</v>
+        <v>482</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>183</v>
+        <v>215</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O63" s="4" t="s">
-        <v>176</v>
+        <v>104</v>
+      </c>
+      <c r="O63" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>63</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>448</v>
+      <c r="B64" s="5" t="s">
+        <v>483</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>18</v>
@@ -4914,39 +5084,133 @@
         <v>19</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>451</v>
+        <v>486</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>291</v>
+        <v>487</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>452</v>
+        <v>488</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>292</v>
+        <v>489</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="M64" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="N64" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="O64" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A65" s="2">
+        <v>64</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>490</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="O65" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A66" s="2">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="L66" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="M66" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="N64" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O64" s="2" t="s">
-        <v>27</v>
+      <c r="N66" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="O66" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="M10:M64">
+    <dataValidation type="list" allowBlank="1" sqref="M10:M66">
       <formula1>"Not Run,Pass,Fail,Blocked,On Hold"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="M2:M64">
+    <dataValidation type="list" allowBlank="1" sqref="M2:M66">
       <formula1>"Not Run,Pass,Fail,Blocked,On Hold"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Implemented Batch 2 of Onboarding Test in production environment
- Automated Batch 2 onboarding flows: password reset confirmations, themed login portals, invalid/role-based logins, and account lockout
- Added onboardingBatch2.page.js and onboardingBatch2.test.js with externalized selectors in C1Selectors.json
- Added test data onboardingB2Data.json and test execution suites onboardingB2Test.json
- Registered OnboardingBatch2 testcases in C1TCRepository.json
- Added npm run script onboardingB2Test_prod in package.json
- Updated manual test case register (_tcdata.js, Onboarding_test_cases.xlsx, Onboarding_test_cases.md)
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="520">
   <si>
     <t>S.No.</t>
   </si>
@@ -333,10 +333,10 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Direct entry to the primary-themed login route.</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Not Run</t>
+    <t>Verified on Production: /login-primary loads with brand logo, primary header, submit button, and footer links.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 2)</t>
   </si>
   <si>
     <t>TST_LAND_TC_9</t>
@@ -361,6 +361,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Direct entry to the secondary-themed login route.</t>
   </si>
   <si>
+    <t>Verified on Production: /login-secondary loads with brand logo, secondary header, submit button, and footer links.</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_5</t>
   </si>
   <si>
@@ -387,6 +390,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_LOGI_TC_5 already clicks Log in and checks the dashboard loads (composed after LOGI_TC_1/2, which type the credentials). Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: user logs in with valid student credentials and lands on dashboard.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 3 via TST_LOGI_TC_1/2/5)</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_7</t>
   </si>
   <si>
@@ -447,6 +456,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Counts as 1 of the 5 attempts before lockout (see TST_LOGI_TC_9) — never run it repeatedly on a shared account; use a disposable one or one whose counter resets on success.</t>
   </si>
   <si>
+    <t>Verified on Production: generic credentials error alert displayed on invalid password and user remains on /login.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 3)</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_9</t>
   </si>
   <si>
@@ -474,6 +489,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. Account is locked for 2 minutes on 5 consecutive wrong password attempts (user confirmed 2026-09-24). Uses dedicated test user cqatestuserforblockDND@mailsac.com.</t>
   </si>
   <si>
+    <t>Verified on Production: 5 consecutive failed login attempts show 5-attempt limit warning, and 6th attempt with valid password is rejected with account temporarily locked message.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 4)</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_10</t>
   </si>
   <si>
@@ -543,6 +564,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_LOGI_TC_6 already clicks Sign up on the login form and checks the page is launched. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not.</t>
   </si>
   <si>
+    <t>Verified on Production: clicking 'Don\'t have an account yet?' navigates to role selection screen (/regoptions).</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 1 via TST_LOGI_TC_6)</t>
+  </si>
+  <si>
     <t>TST_LOGI_TC_11</t>
   </si>
   <si>
@@ -569,6 +596,12 @@
     <t xml:space="preserve">NOT FOR AUTOMATION — marked YELLOW in the source plan (user, 2026-09-24): needs bulk-created username accounts; the first-login gate appears once per account. Manual execution only. Source: OnboardingApp_Test_Plan.xlsx. </t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Not Run</t>
+  </si>
+  <si>
     <t>Manual only — YELLOW in source (not for automation)</t>
   </si>
   <si>
@@ -643,6 +676,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Every admin suite already logs in this way (login.click_login_btn_schoolAdmin in their Before) but none asserts it as a case.</t>
+  </si>
+  <si>
+    <t>Verified on Production: school admin logs in through standard form and reaches /admin/admin/ dashboard.</t>
   </si>
   <si>
     <t>TST_LOGI_TC_15</t>
@@ -745,6 +781,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. EXISTING TC reused (ADR-011 — no duplicate function): TST_APPS_TC_2 already clicks Log out (after TST_APPS_TC_1 opens the menu) and checks the landing page. Phase 1: confirm it asserts this row's Expected Result; extend its assertion if it does not. Knowledge: SOURCE saw logout land on /home OR /login?rurl=… — both are logged-out states; confirm which one the learner gets.</t>
   </si>
   <si>
+    <t>Verified on Production: logging out redirects to landing page with Log in and Sign up options.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 3 via TST_APPS_TC_1/2)</t>
+  </si>
+  <si>
     <t>TST_RESE_TC_6</t>
   </si>
   <si>
@@ -796,6 +838,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. SENDS A REAL RESET E-MAIL to the account (harmless: the password only changes if the link is used). Use a Mailsac-inbox account, not a shared login.</t>
   </si>
   <si>
+    <t>Verified on Production: reset password confirmation screen displays heading "Reset password email sent" and informational body text for registered email.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB2Test_prod (Suite 1)</t>
+  </si>
+  <si>
     <t>TST_RESE_TC_8</t>
   </si>
   <si>
@@ -816,6 +864,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Legend 'Generic reset message': identical by design (no account enumeration), not a bug. 'No reset e-mail is actually sent' can only be checked in the Mailsac inbox.</t>
+  </si>
+  <si>
+    <t>Verified on Production: reset password confirmation screen displays identical generic heading "Reset password email sent" and informational body text for unregistered email (no account enumeration).</t>
   </si>
   <si>
     <t>TST_RESE_TC_4</t>
@@ -2704,11 +2755,11 @@
       <c r="L13" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="M13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="O13" s="2" t="s">
         <v>28</v>
@@ -2749,13 +2800,13 @@
         <v>111</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>28</v>
@@ -2766,13 +2817,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>18</v>
@@ -2781,28 +2832,28 @@
         <v>32</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>105</v>
+        <v>121</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>28</v>
@@ -2813,43 +2864,43 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="O16" s="2" t="s">
         <v>28</v>
@@ -2860,43 +2911,43 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>105</v>
+        <v>141</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="O17" s="2" t="s">
         <v>28</v>
@@ -2907,43 +2958,43 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>105</v>
+        <v>151</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>104</v>
+        <v>152</v>
       </c>
       <c r="O18" s="2" t="s">
         <v>28</v>
@@ -2954,13 +3005,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>18</v>
@@ -2969,28 +3020,28 @@
         <v>19</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="O19" s="2" t="s">
         <v>28</v>
@@ -3001,13 +3052,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>18</v>
@@ -3016,28 +3067,28 @@
         <v>19</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>28</v>
@@ -3048,13 +3099,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>18</v>
@@ -3063,28 +3114,28 @@
         <v>19</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>105</v>
+        <v>175</v>
+      </c>
+      <c r="M21" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>28</v>
@@ -3095,13 +3146,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>18</v>
@@ -3110,31 +3161,31 @@
         <v>19</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -3142,13 +3193,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>18</v>
@@ -3157,31 +3208,31 @@
         <v>19</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -3189,46 +3240,46 @@
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="O24" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="O24" s="4" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -3236,13 +3287,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>18</v>
@@ -3251,28 +3302,28 @@
         <v>32</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>105</v>
+        <v>211</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>104</v>
+        <v>142</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>28</v>
@@ -3283,13 +3334,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>18</v>
@@ -3298,31 +3349,31 @@
         <v>19</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O26" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -3330,13 +3381,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>18</v>
@@ -3345,31 +3396,31 @@
         <v>19</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O27" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -3377,13 +3428,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>18</v>
@@ -3392,31 +3443,31 @@
         <v>19</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="H28" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="O28" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="O28" s="5" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -3424,13 +3475,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>18</v>
@@ -3439,28 +3490,28 @@
         <v>19</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>105</v>
+        <v>241</v>
+      </c>
+      <c r="M29" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>104</v>
+        <v>242</v>
       </c>
       <c r="O29" s="2" t="s">
         <v>28</v>
@@ -3471,43 +3522,43 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>229</v>
+        <v>243</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>231</v>
+        <v>245</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>28</v>
@@ -3518,13 +3569,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>18</v>
@@ -3533,28 +3584,28 @@
         <v>32</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>105</v>
+        <v>259</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>104</v>
+        <v>260</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>28</v>
@@ -3565,43 +3616,43 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>105</v>
+        <v>268</v>
+      </c>
+      <c r="M32" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>104</v>
+        <v>260</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>28</v>
@@ -3612,13 +3663,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>18</v>
@@ -3627,28 +3678,28 @@
         <v>19</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="O33" s="2" t="s">
         <v>28</v>
@@ -3659,13 +3710,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>18</v>
@@ -3674,28 +3725,28 @@
         <v>32</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>265</v>
+        <v>282</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O34" s="2" t="s">
         <v>28</v>
@@ -3706,13 +3757,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>266</v>
+        <v>283</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>267</v>
+        <v>284</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>268</v>
+        <v>285</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>18</v>
@@ -3721,28 +3772,28 @@
         <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>269</v>
+        <v>286</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>270</v>
+        <v>287</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>271</v>
+        <v>288</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>272</v>
+        <v>289</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>273</v>
+        <v>290</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>28</v>
@@ -3753,13 +3804,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>274</v>
+        <v>291</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>275</v>
+        <v>292</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>276</v>
+        <v>293</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>18</v>
@@ -3768,28 +3819,28 @@
         <v>32</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>277</v>
+        <v>294</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>279</v>
+        <v>296</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>280</v>
+        <v>297</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>281</v>
+        <v>298</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O36" s="2" t="s">
         <v>28</v>
@@ -3800,13 +3851,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>282</v>
+        <v>299</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>276</v>
+        <v>293</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>18</v>
@@ -3815,28 +3866,28 @@
         <v>32</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>284</v>
+        <v>301</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>285</v>
+        <v>302</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>286</v>
+        <v>303</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>288</v>
+        <v>305</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O37" s="2" t="s">
         <v>28</v>
@@ -3847,13 +3898,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>289</v>
+        <v>306</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>290</v>
+        <v>307</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>291</v>
+        <v>308</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>18</v>
@@ -3862,28 +3913,28 @@
         <v>32</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>293</v>
+        <v>310</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>294</v>
+        <v>311</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>295</v>
+        <v>312</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>296</v>
+        <v>313</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O38" s="2" t="s">
         <v>28</v>
@@ -3894,13 +3945,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>297</v>
+        <v>314</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>299</v>
+        <v>316</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>18</v>
@@ -3912,25 +3963,25 @@
         <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>300</v>
+        <v>317</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>301</v>
+        <v>318</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>302</v>
+        <v>319</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>303</v>
+        <v>320</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="O39" s="2" t="s">
         <v>28</v>
@@ -3941,13 +3992,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>305</v>
+        <v>322</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>307</v>
+        <v>324</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>18</v>
@@ -3956,28 +4007,28 @@
         <v>32</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>309</v>
+        <v>326</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>310</v>
+        <v>327</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>311</v>
+        <v>328</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>312</v>
+        <v>329</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>313</v>
+        <v>330</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>28</v>
@@ -3988,13 +4039,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>314</v>
+        <v>331</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>316</v>
+        <v>333</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>18</v>
@@ -4003,28 +4054,28 @@
         <v>19</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>317</v>
+        <v>334</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>310</v>
+        <v>327</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>318</v>
+        <v>335</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>319</v>
+        <v>336</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>28</v>
@@ -4035,13 +4086,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>320</v>
+        <v>337</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>321</v>
+        <v>338</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>18</v>
@@ -4050,28 +4101,28 @@
         <v>32</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>323</v>
+        <v>340</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>325</v>
+        <v>342</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>326</v>
+        <v>343</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>327</v>
+        <v>344</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>328</v>
+        <v>345</v>
       </c>
       <c r="O42" s="2" t="s">
         <v>28</v>
@@ -4082,13 +4133,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>329</v>
+        <v>346</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>330</v>
+        <v>347</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>331</v>
+        <v>348</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>18</v>
@@ -4097,28 +4148,28 @@
         <v>19</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>332</v>
+        <v>349</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>334</v>
+        <v>351</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="O43" s="2" t="s">
         <v>28</v>
@@ -4129,13 +4180,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>335</v>
+        <v>352</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>336</v>
+        <v>353</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>337</v>
+        <v>354</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>18</v>
@@ -4144,28 +4195,28 @@
         <v>32</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>338</v>
+        <v>355</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>339</v>
+        <v>356</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>340</v>
+        <v>357</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>341</v>
+        <v>358</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>342</v>
+        <v>359</v>
       </c>
       <c r="O44" s="2" t="s">
         <v>28</v>
@@ -4176,43 +4227,43 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>344</v>
+        <v>361</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>345</v>
+        <v>362</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>347</v>
+        <v>364</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>348</v>
+        <v>365</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>349</v>
+        <v>366</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>350</v>
+        <v>367</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>351</v>
+        <v>368</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>342</v>
+        <v>359</v>
       </c>
       <c r="O45" s="2" t="s">
         <v>28</v>
@@ -4223,43 +4274,43 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>352</v>
+        <v>369</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>353</v>
+        <v>370</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>354</v>
+        <v>371</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>355</v>
+        <v>372</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>356</v>
+        <v>373</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>357</v>
+        <v>374</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>358</v>
+        <v>375</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>359</v>
+        <v>376</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>360</v>
+        <v>377</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>342</v>
+        <v>359</v>
       </c>
       <c r="O46" s="2" t="s">
         <v>28</v>
@@ -4270,13 +4321,13 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>361</v>
+        <v>378</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>362</v>
+        <v>379</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>363</v>
+        <v>380</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>18</v>
@@ -4285,28 +4336,28 @@
         <v>19</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>364</v>
+        <v>381</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>365</v>
+        <v>382</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>366</v>
+        <v>383</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>367</v>
+        <v>384</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>368</v>
+        <v>385</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>369</v>
+        <v>386</v>
       </c>
       <c r="O47" s="2" t="s">
         <v>28</v>
@@ -4317,13 +4368,13 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>372</v>
+        <v>389</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>18</v>
@@ -4332,28 +4383,28 @@
         <v>32</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>374</v>
+        <v>391</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>375</v>
+        <v>392</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>376</v>
+        <v>393</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>377</v>
+        <v>394</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O48" s="2" t="s">
         <v>28</v>
@@ -4364,43 +4415,43 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>378</v>
+        <v>395</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>379</v>
+        <v>396</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>380</v>
+        <v>397</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>381</v>
+        <v>398</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>382</v>
+        <v>399</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>384</v>
+        <v>401</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>385</v>
+        <v>402</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>342</v>
+        <v>359</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>28</v>
@@ -4411,13 +4462,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>386</v>
+        <v>403</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>387</v>
+        <v>404</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>388</v>
+        <v>405</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>18</v>
@@ -4426,28 +4477,28 @@
         <v>32</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>389</v>
+        <v>406</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>390</v>
+        <v>407</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>391</v>
+        <v>408</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>392</v>
+        <v>409</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>28</v>
@@ -4458,43 +4509,43 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>393</v>
+        <v>410</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>394</v>
+        <v>411</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>395</v>
+        <v>412</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>396</v>
+        <v>413</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>397</v>
+        <v>414</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>398</v>
+        <v>415</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>399</v>
+        <v>416</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>400</v>
+        <v>417</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>28</v>
@@ -4505,13 +4556,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>401</v>
+        <v>418</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>402</v>
+        <v>419</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>18</v>
@@ -4520,28 +4571,28 @@
         <v>32</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>404</v>
+        <v>421</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>405</v>
+        <v>422</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>406</v>
+        <v>423</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>407</v>
+        <v>424</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>28</v>
@@ -4552,43 +4603,43 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>408</v>
+        <v>425</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>410</v>
+        <v>427</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>411</v>
+        <v>428</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>412</v>
+        <v>429</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>413</v>
+        <v>430</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>414</v>
+        <v>431</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>415</v>
+        <v>432</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O53" s="2" t="s">
         <v>28</v>
@@ -4599,13 +4650,13 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>416</v>
+        <v>433</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>417</v>
+        <v>434</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>418</v>
+        <v>435</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>18</v>
@@ -4614,28 +4665,28 @@
         <v>32</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>419</v>
+        <v>436</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>420</v>
+        <v>437</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>421</v>
+        <v>438</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>422</v>
+        <v>439</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>423</v>
+        <v>440</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>28</v>
@@ -4646,43 +4697,43 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>424</v>
+        <v>441</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>425</v>
+        <v>442</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>426</v>
+        <v>443</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>427</v>
+        <v>444</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>428</v>
+        <v>445</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>429</v>
+        <v>446</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>430</v>
+        <v>447</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O55" s="2" t="s">
         <v>28</v>
@@ -4693,13 +4744,13 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>431</v>
+        <v>448</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>432</v>
+        <v>449</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>433</v>
+        <v>450</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>18</v>
@@ -4708,28 +4759,28 @@
         <v>32</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>434</v>
+        <v>451</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>435</v>
+        <v>452</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>436</v>
+        <v>453</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>437</v>
+        <v>454</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>438</v>
+        <v>455</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>28</v>
@@ -4740,13 +4791,13 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>439</v>
+        <v>456</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>440</v>
+        <v>457</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>441</v>
+        <v>458</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>18</v>
@@ -4755,28 +4806,28 @@
         <v>32</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>442</v>
+        <v>459</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>443</v>
+        <v>460</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>444</v>
+        <v>461</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>445</v>
+        <v>462</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>446</v>
+        <v>463</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>28</v>
@@ -4787,13 +4838,13 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>447</v>
+        <v>464</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>448</v>
+        <v>465</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>449</v>
+        <v>466</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>18</v>
@@ -4802,28 +4853,28 @@
         <v>19</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>450</v>
+        <v>467</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>451</v>
+        <v>468</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>453</v>
+        <v>470</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>454</v>
+        <v>471</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>28</v>
@@ -4834,13 +4885,13 @@
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>455</v>
+        <v>472</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>456</v>
+        <v>473</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>457</v>
+        <v>474</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>18</v>
@@ -4852,28 +4903,28 @@
         <v>20</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>458</v>
+        <v>475</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>459</v>
+        <v>476</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O59" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
@@ -4881,13 +4932,13 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>460</v>
+        <v>477</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>461</v>
+        <v>478</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>462</v>
+        <v>479</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>18</v>
@@ -4896,31 +4947,31 @@
         <v>19</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>463</v>
+        <v>480</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>464</v>
+        <v>481</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O60" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
@@ -4928,13 +4979,13 @@
         <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>465</v>
+        <v>482</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>466</v>
+        <v>483</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>467</v>
+        <v>484</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>18</v>
@@ -4943,31 +4994,31 @@
         <v>19</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>468</v>
+        <v>485</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O61" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
@@ -4975,13 +5026,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>471</v>
+        <v>488</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>472</v>
+        <v>489</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>473</v>
+        <v>490</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>18</v>
@@ -4990,31 +5041,31 @@
         <v>19</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>474</v>
+        <v>491</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>475</v>
+        <v>492</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
@@ -5022,13 +5073,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>476</v>
+        <v>493</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>477</v>
+        <v>494</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>478</v>
+        <v>495</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>18</v>
@@ -5037,31 +5088,31 @@
         <v>19</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>479</v>
+        <v>496</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>480</v>
+        <v>497</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>481</v>
+        <v>498</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>482</v>
+        <v>499</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O63" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
@@ -5069,13 +5120,13 @@
         <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>483</v>
+        <v>500</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>484</v>
+        <v>501</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>485</v>
+        <v>502</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>18</v>
@@ -5084,31 +5135,31 @@
         <v>19</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>487</v>
+        <v>504</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>488</v>
+        <v>505</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O64" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
@@ -5116,13 +5167,13 @@
         <v>64</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>490</v>
+        <v>507</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>492</v>
+        <v>509</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>18</v>
@@ -5131,31 +5182,31 @@
         <v>19</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>493</v>
+        <v>510</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>494</v>
+        <v>511</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>495</v>
+        <v>512</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>496</v>
+        <v>513</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="M65" s="2" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>104</v>
+        <v>185</v>
       </c>
       <c r="O65" s="5" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
@@ -5163,13 +5214,13 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>497</v>
+        <v>514</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>498</v>
+        <v>515</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>499</v>
+        <v>516</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>18</v>
@@ -5178,28 +5229,28 @@
         <v>19</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>332</v>
+        <v>349</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>333</v>
+        <v>350</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="M66" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>342</v>
+        <v>359</v>
       </c>
       <c r="O66" s="2" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
Implemented Batch 3 of Onboarding Test in production environment
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/Onboarding/Onboarding_test_cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="544">
   <si>
     <t>S.No.</t>
   </si>
@@ -916,6 +916,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. CHANGES A REAL ACCOUNT'S PASSWORD — use a disposable account (e.g. one created by the signup suite in the same run), never a shared fixture. Mail handling as mailsacUI.openVerificationLink (sandboxed mail iframe, follow the link on the same page — c1-core-shared.md §A5/§B3). The reset link host may be the same login.comprodls.com host whose thor certificate is expired [ASSUMED — check].</t>
   </si>
   <si>
+    <t>Verified on Production: password reset requested, link extracted from Mailsac inbox, new password saved and confirmed via modal dialog, and user successfully logs in with new password.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 5)</t>
+  </si>
+  <si>
     <t>TST_RESE_TC_10</t>
   </si>
   <si>
@@ -943,6 +949,9 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. OVERLAP: the source's TC_FPWD_005 already ends with this login (its steps 5–6). Kept as its own row because the source has it; see Open items — the automation may compose LOGI_TC_1/2/5 with the new password instead of a new function.</t>
   </si>
   <si>
+    <t>Verified on Production: user logs out from active session, enters credentials with newly reset password on /login, and reaches role dashboard.</t>
+  </si>
+  <si>
     <t>TST_CREA_TC_31</t>
   </si>
   <si>
@@ -969,6 +978,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. First half of the source row; the student's first login with the temporary password is TST_LOGI_TC_18. CHANGES A REAL STUDENT'S PASSWORD — disposable student only. Module CREA = the teacher class page object (createNewClass.page.js); if Phase 1 finds the roster lives on another page object, re-code before automating. Confirmation copy after submit is [ASSUMED] (not in the source).</t>
+  </si>
+  <si>
+    <t>Verified on Production: Teacher opens class roster on Class data tab, locates student Actions menu, and verifies options to change password and manage student.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test (Suite 8 via TST_CREA_TC_31)</t>
   </si>
   <si>
     <t>TST_LOGI_TC_18</t>
@@ -994,7 +1009,7 @@
 3. The student can log in again with the new, self-set password.</t>
   </si>
   <si>
-    <t>Source: OnboardingApp_Test_Plan.xlsx. Serves BOTH TC_RESETPW_001 and TC_RESETPW_002 (same screen, different staff entry). Legend 'Password reset caveat': the same Gigya temporary-password screen-set as an Admin resetting their own password.</t>
+    <t>Source: OnboardingApp_Test_Plan.xlsx. Serves BOTH TC_RESETPW_001 and TC_RESETPW_002 (same screen, different staff entry). Out of automation scope per user instruction.</t>
   </si>
   <si>
     <t>TST_SPRF_TC_24</t>
@@ -1023,6 +1038,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. [ASSUMED] entry point — the source's Legend says it was "taken from existing documentation … not independently re-verified live". OVERLAP to settle in Phase 1: the Students register already has TST_SPRF_TC_8 (admin sets a NEW password via View profile &gt; Manage account &gt; Password tab) and TST_SPRF_TC_23 (learner signs in with it). This row differs by the row Action Menu entry and the TEMPORARY-password first-login screen — confirm live that these are two different flows before automating. CHANGES A REAL STUDENT'S PASSWORD — disposable student only.</t>
+  </si>
+  <si>
+    <t>Verified on Production: School admin navigates to Learners tab, accesses learner profile, opens Manage learner profile, sets temporary password, and submits update.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test (Suite 8 via TST_SPRF_TC_24)</t>
   </si>
   <si>
     <t>TST_SNUP_TC_65</t>
@@ -1283,6 +1304,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. CREATES REAL DATA (a platform account) — ADR-021: needs the user's OK on a shared environment; place in a data-creating suite. Thor: the e-mail verification link host has an EXPIRED certificate (c1-core-shared.md §A4) — the verify step is blocked on thor until renewed; production works. New assertion = the locked, pre-filled Location. Account creation/verification reuse existing TST_SNUP_TC_60 (submit → pending screen), TST_SNUP_TC_61 (Mailsac link), TST_SNUP_TC_64 (learner welcome).</t>
+  </si>
+  <si>
+    <t>Verified on Production: Location is locked to pre-filled value from age check, user completes registration form, verifies account via Mailsac link, and successfully accesses Learner dashboard.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 2)</t>
   </si>
   <si>
     <t>TST_SNUP_TC_76</t>
@@ -1342,6 +1369,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. CREATES REAL DATA (a platform account) — ADR-021: needs the user's OK on a shared environment; place in a data-creating suite. Thor: the e-mail verification link host has an EXPIRED certificate (c1-core-shared.md §A4) — the verify step is blocked on thor until renewed; production works. New assertion = the Teacher form's fields / no age gate. Creation and verification reuse existing TST_SNUP_TC_60, TST_SNUP_TC_61, TST_SNUP_TC_62 (tour + "Complete account set up").</t>
   </si>
   <si>
+    <t>Verified on Production: Teacher registration form opens directly with no age gate, user completes registration, verifies account via Mailsac link, and reaches Teacher dashboard / complete account setup prompt.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 3)</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_77</t>
   </si>
   <si>
@@ -1371,6 +1404,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Side-effect free. Terms checkbox id differs by env (thor #legal-checkbox-1, prod #teacher-checkbox-1 — onboarding.md §A3).</t>
+  </si>
+  <si>
+    <t>Verified on Production: required-field errors ('This field is required') shown for First name, Last name, Location; 'E-mail address is invalid.' for Work email; 'Password does not meet complexity requirements' for weak password; Terms alert displayed when unchecked.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 1)</t>
   </si>
   <si>
     <t>TST_SNUP_TC_74</t>
@@ -1401,6 +1440,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. CREATES REAL DATA (a platform account) — ADR-021: needs the user's OK on a shared environment; place in a data-creating suite. Thor: the e-mail verification link host has an EXPIRED certificate (c1-core-shared.md §A4) — the verify step is blocked on thor until renewed; production works. Resolves onboarding.md §A2's [ASSUMED] Parent row. Creation/verification reuse TST_SNUP_TC_60/61; the parent dashboard assertion is new.</t>
   </si>
   <si>
+    <t>Verified on Production: Parent registration form includes age 18+ / guardian consent checkbox, user completes registration, verifies account via Mailsac link, and reaches Parent dashboard.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 4)</t>
+  </si>
+  <si>
     <t>TST_SNUP_TC_75</t>
   </si>
   <si>
@@ -1425,6 +1470,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Any message shown for the missing checkbox is not stated in the source — capture it verbatim in Phase 1 [ASSUMED]. Side-effect free if the form really does not submit; use a {{run.*}} e-mail anyway in case it does.</t>
+  </si>
+  <si>
+    <t>Verified on Production: Parent form does not submit without guardian consent, user remains on /register-parent, and parental checkbox highlights with error state (.parent-error).</t>
   </si>
   <si>
     <t>TST_PCHD_TC_1</t>
@@ -1458,6 +1506,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. PROPOSED module PCHD — no parent/child page object exists yet (migration plan U20, K19: the child form sits in a Gigya #child-iframe). CREATES A CHILD ACCOUNT. SOURCE reported child creation FAILING ON THOR [2026] — Phase 1 must check; if still failing, mark Blocked there (unblock: product fix or run on another env with the user's OK).</t>
   </si>
   <si>
+    <t>Verified on Production: Parent creates child account from 'My children', completes embedded panel details with consent checkbox, enters child username &amp; password, and receives account created confirmation with username.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test_prod (Suite 6)</t>
+  </si>
+  <si>
     <t>TST_PCHD_TC_2</t>
   </si>
   <si>
@@ -1478,6 +1532,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Exact inline error copy is not in the source — capture verbatim in Phase 1 [ASSUMED]. Side-effect free.</t>
+  </si>
+  <si>
+    <t>Verified on Production: on 'Create my child's account' blank submission displays required-field errors ('This field is required', 'This field is required (Month and Year)'), and form stays blocked on Subscreen 1 without ticking the consent checkbox.</t>
   </si>
   <si>
     <t>TST_PCHD_TC_3</t>
@@ -1505,6 +1562,9 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Depends on TST_PCHD_TC_1 in the same run.</t>
+  </si>
+  <si>
+    <t>Verified on Production: newly created child account logs in with username and password on /login, and successfully reaches the Learner dashboard ('Learner dashboard | Cambridge One').</t>
   </si>
   <si>
     <t>TST_INVI_TC_14</t>
@@ -1539,6 +1599,12 @@
     <t>Source: OnboardingApp_Test_Plan.xlsx. CREATES REAL DATA (a platform account) — ADR-021: needs the user's OK on a shared environment; place in a data-creating suite. Needs a teacher + class and an invite (reuse TST_CREA_TC_19–24 for the invite). Module INVI (invitation flow); if Phase 1 finds the invite signup form is the signup page object, re-code to SNUP before automating. Legend: invite signup has NO age gate.</t>
   </si>
   <si>
+    <t>Verified on Production: Teacher invites unregistered student, invitee opens 'View invite' link from Mailsac email, completes registration with prefilled email, verifies account via Mailsac, and reaches dashboard.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test (Suite 7 via TST_INVI_TC_14)</t>
+  </si>
+  <si>
     <t>TST_INVI_TC_15</t>
   </si>
   <si>
@@ -1561,6 +1627,12 @@
   </si>
   <si>
     <t>Source: OnboardingApp_Test_Plan.xlsx. Existing INVI_TC_1–6 cover accepting the invite from the in-app bell; this is the e-mail link path. Each run leaves a pending invite in the class (migration plan Q4).</t>
+  </si>
+  <si>
+    <t>Verified on Production: Teacher invites registered learner, learner opens 'View invite' link while logged in, and lands directly on their learner dashboard.</t>
+  </si>
+  <si>
+    <t>Automated in onboardingB3Test (Suite 7 via TST_INVI_TC_15)</t>
   </si>
   <si>
     <t>TST_LOGI_TC_19</t>
@@ -3740,13 +3812,13 @@
         <v>282</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>186</v>
+        <v>283</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>185</v>
+        <v>284</v>
       </c>
       <c r="O34" s="2" t="s">
         <v>28</v>
@@ -3757,13 +3829,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>18</v>
@@ -3772,28 +3844,28 @@
         <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>186</v>
+        <v>293</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>185</v>
+        <v>284</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>28</v>
@@ -3804,13 +3876,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>18</v>
@@ -3819,28 +3891,28 @@
         <v>32</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>186</v>
+        <v>302</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>185</v>
+        <v>303</v>
       </c>
       <c r="O36" s="2" t="s">
         <v>28</v>
@@ -3850,14 +3922,14 @@
       <c r="A37" s="2">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>299</v>
+      <c r="B37" s="4" t="s">
+        <v>304</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>18</v>
@@ -3866,19 +3938,19 @@
         <v>32</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>185</v>
@@ -3889,8 +3961,8 @@
       <c r="N37" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="O37" s="2" t="s">
-        <v>28</v>
+      <c r="O37" s="4" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
@@ -3898,13 +3970,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>18</v>
@@ -3913,28 +3985,28 @@
         <v>32</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>186</v>
+        <v>319</v>
+      </c>
+      <c r="M38" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>185</v>
+        <v>320</v>
       </c>
       <c r="O38" s="2" t="s">
         <v>28</v>
@@ -3945,13 +4017,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>18</v>
@@ -3963,25 +4035,25 @@
         <v>20</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="O39" s="2" t="s">
         <v>28</v>
@@ -3992,13 +4064,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>18</v>
@@ -4007,28 +4079,28 @@
         <v>32</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>28</v>
@@ -4039,13 +4111,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>18</v>
@@ -4054,28 +4126,28 @@
         <v>19</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="J41" s="2" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>249</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>28</v>
@@ -4086,13 +4158,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>18</v>
@@ -4101,28 +4173,28 @@
         <v>32</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="O42" s="2" t="s">
         <v>28</v>
@@ -4133,13 +4205,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>18</v>
@@ -4148,28 +4220,28 @@
         <v>19</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>249</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="O43" s="2" t="s">
         <v>28</v>
@@ -4180,13 +4252,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>18</v>
@@ -4195,28 +4267,28 @@
         <v>32</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="O44" s="2" t="s">
         <v>28</v>
@@ -4227,13 +4299,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>126</v>
@@ -4242,28 +4314,28 @@
         <v>32</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="O45" s="2" t="s">
         <v>28</v>
@@ -4274,43 +4346,43 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>32</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="O46" s="2" t="s">
         <v>28</v>
@@ -4321,13 +4393,13 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>18</v>
@@ -4336,28 +4408,28 @@
         <v>19</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="O47" s="2" t="s">
         <v>28</v>
@@ -4368,13 +4440,13 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>18</v>
@@ -4383,28 +4455,28 @@
         <v>32</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M48" s="2" t="s">
-        <v>186</v>
+        <v>402</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>185</v>
+        <v>403</v>
       </c>
       <c r="O48" s="2" t="s">
         <v>28</v>
@@ -4415,13 +4487,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>396</v>
+        <v>405</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>397</v>
+        <v>406</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>126</v>
@@ -4430,28 +4502,28 @@
         <v>32</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>398</v>
+        <v>407</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>400</v>
+        <v>409</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>401</v>
+        <v>410</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>28</v>
@@ -4462,13 +4534,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>403</v>
+        <v>412</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>404</v>
+        <v>413</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>405</v>
+        <v>414</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>18</v>
@@ -4477,28 +4549,28 @@
         <v>32</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>406</v>
+        <v>415</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>407</v>
+        <v>416</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>408</v>
+        <v>417</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>409</v>
+        <v>418</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>186</v>
+        <v>419</v>
+      </c>
+      <c r="M50" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>185</v>
+        <v>420</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>28</v>
@@ -4509,13 +4581,13 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>126</v>
@@ -4524,28 +4596,28 @@
         <v>32</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>413</v>
+        <v>424</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>414</v>
+        <v>425</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>415</v>
+        <v>426</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>416</v>
+        <v>427</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>417</v>
+        <v>428</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>186</v>
+        <v>429</v>
+      </c>
+      <c r="M51" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>185</v>
+        <v>430</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>28</v>
@@ -4556,13 +4628,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>418</v>
+        <v>431</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>419</v>
+        <v>432</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>18</v>
@@ -4571,28 +4643,28 @@
         <v>32</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>421</v>
+        <v>434</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>422</v>
+        <v>435</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>423</v>
+        <v>436</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>424</v>
+        <v>437</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>186</v>
+        <v>438</v>
+      </c>
+      <c r="M52" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>185</v>
+        <v>439</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>28</v>
@@ -4603,13 +4675,13 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>126</v>
@@ -4618,28 +4690,28 @@
         <v>32</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>428</v>
+        <v>443</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>429</v>
+        <v>444</v>
       </c>
       <c r="I53" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="M53" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N53" s="2" t="s">
         <v>430</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="K53" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="N53" s="2" t="s">
-        <v>185</v>
       </c>
       <c r="O53" s="2" t="s">
         <v>28</v>
@@ -4650,13 +4722,13 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>18</v>
@@ -4665,28 +4737,28 @@
         <v>32</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>440</v>
+        <v>456</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M54" s="2" t="s">
-        <v>186</v>
+        <v>457</v>
+      </c>
+      <c r="M54" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>185</v>
+        <v>458</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>28</v>
@@ -4697,13 +4769,13 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>441</v>
+        <v>459</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>443</v>
+        <v>461</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>126</v>
@@ -4712,28 +4784,28 @@
         <v>19</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>444</v>
+        <v>462</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>445</v>
+        <v>463</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>446</v>
+        <v>464</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>447</v>
+        <v>465</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>186</v>
+        <v>466</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>185</v>
+        <v>458</v>
       </c>
       <c r="O55" s="2" t="s">
         <v>28</v>
@@ -4744,13 +4816,13 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>448</v>
+        <v>467</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>18</v>
@@ -4759,28 +4831,28 @@
         <v>32</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>452</v>
+        <v>471</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>453</v>
+        <v>472</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>454</v>
+        <v>473</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>455</v>
+        <v>474</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>186</v>
+        <v>475</v>
+      </c>
+      <c r="M56" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>185</v>
+        <v>458</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>28</v>
@@ -4791,13 +4863,13 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>458</v>
+        <v>478</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>18</v>
@@ -4806,28 +4878,28 @@
         <v>32</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>459</v>
+        <v>479</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>461</v>
+        <v>481</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M57" s="2" t="s">
-        <v>186</v>
+        <v>484</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>185</v>
+        <v>485</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>28</v>
@@ -4838,13 +4910,13 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>464</v>
+        <v>486</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>465</v>
+        <v>487</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>466</v>
+        <v>488</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>18</v>
@@ -4853,28 +4925,28 @@
         <v>19</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>467</v>
+        <v>489</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>468</v>
+        <v>490</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>469</v>
+        <v>491</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>470</v>
+        <v>492</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>471</v>
+        <v>493</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>186</v>
+        <v>494</v>
+      </c>
+      <c r="M58" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>185</v>
+        <v>495</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>28</v>
@@ -4885,13 +4957,13 @@
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>472</v>
+        <v>496</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>473</v>
+        <v>497</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>474</v>
+        <v>498</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>18</v>
@@ -4903,13 +4975,13 @@
         <v>20</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>475</v>
+        <v>499</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>476</v>
+        <v>500</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>227</v>
@@ -4932,13 +5004,13 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>477</v>
+        <v>501</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>478</v>
+        <v>502</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>479</v>
+        <v>503</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>18</v>
@@ -4947,16 +5019,16 @@
         <v>19</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>480</v>
+        <v>504</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>481</v>
+        <v>505</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>227</v>
@@ -4979,13 +5051,13 @@
         <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>482</v>
+        <v>506</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>483</v>
+        <v>507</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>484</v>
+        <v>508</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>18</v>
@@ -4994,16 +5066,16 @@
         <v>19</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>485</v>
+        <v>509</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>486</v>
+        <v>510</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>487</v>
+        <v>511</v>
       </c>
       <c r="K61" s="2" t="s">
         <v>227</v>
@@ -5026,13 +5098,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>488</v>
+        <v>512</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>489</v>
+        <v>513</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>490</v>
+        <v>514</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>18</v>
@@ -5041,16 +5113,16 @@
         <v>19</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>491</v>
+        <v>515</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>22</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>492</v>
+        <v>516</v>
       </c>
       <c r="K62" s="2" t="s">
         <v>227</v>
@@ -5073,13 +5145,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>493</v>
+        <v>517</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>494</v>
+        <v>518</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>495</v>
+        <v>519</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>18</v>
@@ -5088,16 +5160,16 @@
         <v>19</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>496</v>
+        <v>520</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>497</v>
+        <v>521</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>498</v>
+        <v>522</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>499</v>
+        <v>523</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>227</v>
@@ -5120,13 +5192,13 @@
         <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>500</v>
+        <v>524</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>501</v>
+        <v>525</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>502</v>
+        <v>526</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>18</v>
@@ -5135,16 +5207,16 @@
         <v>19</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>503</v>
+        <v>527</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>504</v>
+        <v>528</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>505</v>
+        <v>529</v>
       </c>
       <c r="J64" s="2" t="s">
-        <v>506</v>
+        <v>530</v>
       </c>
       <c r="K64" s="2" t="s">
         <v>227</v>
@@ -5167,13 +5239,13 @@
         <v>64</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>507</v>
+        <v>531</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>508</v>
+        <v>532</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>509</v>
+        <v>533</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>18</v>
@@ -5182,16 +5254,16 @@
         <v>19</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>510</v>
+        <v>534</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>511</v>
+        <v>535</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>512</v>
+        <v>536</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>513</v>
+        <v>537</v>
       </c>
       <c r="K65" s="2" t="s">
         <v>227</v>
@@ -5214,13 +5286,13 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>514</v>
+        <v>538</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>515</v>
+        <v>539</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>516</v>
+        <v>540</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>18</v>
@@ -5229,28 +5301,28 @@
         <v>19</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>517</v>
+        <v>541</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>518</v>
+        <v>542</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="K66" s="2" t="s">
         <v>249</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>519</v>
+        <v>543</v>
       </c>
       <c r="M66" s="3" t="s">
         <v>26</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="O66" s="2" t="s">
         <v>28</v>

</xml_diff>